<commit_message>
feat: integrate Selenium Grid with GitHub Actions CI for cross-browser parallel execution
</commit_message>
<xml_diff>
--- a/src/test/resources/RegistrationData.xlsx
+++ b/src/test/resources/RegistrationData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/FC18120534C56AB2/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\OpenCart(1)\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FF8C6BC-5914-4997-85B0-D584FE309A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A05D6D8-64DD-4F3F-8137-DB2CB31FAE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{4648B6AC-A5E7-4088-BDE6-266068846D05}"/>
   </bookViews>
@@ -248,10 +248,10 @@
     <t>Brown</t>
   </si>
   <si>
-    <t>short</t>
-  </si>
-  <si>
     <t>Password must be between 4 and 20 characters!</t>
+  </si>
+  <si>
+    <t>sh</t>
   </si>
 </sst>
 </file>
@@ -757,7 +757,7 @@
         <v>28</v>
       </c>
       <c r="E5" s="2">
-        <v>123</v>
+        <v>13</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>29</v>
@@ -783,10 +783,10 @@
         <v>5559876543</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>